<commit_message>
Add new workout example PDF and update evaluation report Excel file
- Introduced a new PDF file titled `workout example.pdf` to provide additional resources for the project.
- Updated the existing Excel file `evaluation_report_drf.xlsx` to reflect the latest evaluation metrics and findings, enhancing data analysis capabilities.
</commit_message>
<xml_diff>
--- a/docs/data_evaluation-deepseek-routing-3.1flash-lite-all/django-rest-framework/evaluation_report_drf.xlsx
+++ b/docs/data_evaluation-deepseek-routing-3.1flash-lite-all/django-rest-framework/evaluation_report_drf.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sagundevkota/Documents/opensource/hierarchical-rag/data_evaluation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sagundevkota/Documents/opensource/hierarchical-rag/docs/data_evaluation-deepseek-routing-3.1flash-lite-all/django-rest-framework/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{227989A2-0473-394F-A737-BE26BD88209B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83C0526F-42FF-4D44-9768-1D0624194C89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -205,10 +205,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -268,8 +267,13 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Context Precision</a:t>
+              <a:t>Context Precision by Question</a:t>
             </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Type (higher is better)</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -590,6 +594,7 @@
         <c:axId val="1927448016"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="1.2"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -760,8 +765,13 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Context Recall</a:t>
+              <a:t>Context Recall by Question Type (higher</a:t>
             </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> is better)</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -8523,10 +8533,10 @@
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>177800</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>315468</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>175768</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8553,16 +8563,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>317500</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>12700</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>101600</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>25400</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>10668</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>10668</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -9648,7 +9658,7 @@
       <c r="F11" s="1">
         <v>0.96</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11">
         <v>0.59160000000000001</v>
       </c>
       <c r="H11">
@@ -9787,26 +9797,26 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>20</v>
       </c>
     </row>
@@ -9814,15 +9824,15 @@
       <c r="A5" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="5">
         <f>SUMIFS('RAG Comparison'!$C:$C,'RAG Comparison'!$A:$A,$A5,'RAG Comparison'!$B:$B,B$4)</f>
         <v>0.91610000000000003</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="5">
         <f>SUMIFS('RAG Comparison'!$C:$C,'RAG Comparison'!$A:$A,$A5,'RAG Comparison'!$B:$B,C$4)</f>
         <v>0.74719999999999998</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="5">
         <f>SUMIFS('RAG Comparison'!$C:$C,'RAG Comparison'!$A:$A,$A5,'RAG Comparison'!$B:$B,D$4)</f>
         <v>0.74970000000000003</v>
       </c>
@@ -9831,15 +9841,15 @@
       <c r="A6" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="5">
         <f>SUMIFS('RAG Comparison'!$C:$C,'RAG Comparison'!$A:$A,$A6,'RAG Comparison'!$B:$B,B$4)</f>
         <v>0.84419999999999995</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="5">
         <f>SUMIFS('RAG Comparison'!$C:$C,'RAG Comparison'!$A:$A,$A6,'RAG Comparison'!$B:$B,C$4)</f>
         <v>0.64539999999999997</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="5">
         <f>SUMIFS('RAG Comparison'!$C:$C,'RAG Comparison'!$A:$A,$A6,'RAG Comparison'!$B:$B,D$4)</f>
         <v>0.67290000000000005</v>
       </c>
@@ -9848,15 +9858,15 @@
       <c r="A7" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="5">
         <f>SUMIFS('RAG Comparison'!$C:$C,'RAG Comparison'!$A:$A,$A7,'RAG Comparison'!$B:$B,B$4)</f>
         <v>0.88839999999999997</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="5">
         <f>SUMIFS('RAG Comparison'!$C:$C,'RAG Comparison'!$A:$A,$A7,'RAG Comparison'!$B:$B,C$4)</f>
         <v>0.44779999999999998</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="5">
         <f>SUMIFS('RAG Comparison'!$C:$C,'RAG Comparison'!$A:$A,$A7,'RAG Comparison'!$B:$B,D$4)</f>
         <v>0.53449999999999998</v>
       </c>
@@ -9865,35 +9875,35 @@
       <c r="A8" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="5">
         <f>SUMIFS('RAG Comparison'!$C:$C,'RAG Comparison'!$A:$A,$A8,'RAG Comparison'!$B:$B,B$4)</f>
         <v>0.92610000000000003</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="5">
         <f>SUMIFS('RAG Comparison'!$C:$C,'RAG Comparison'!$A:$A,$A8,'RAG Comparison'!$B:$B,C$4)</f>
         <v>0.76180000000000003</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="5">
         <f>SUMIFS('RAG Comparison'!$C:$C,'RAG Comparison'!$A:$A,$A8,'RAG Comparison'!$B:$B,D$4)</f>
         <v>0.72760000000000002</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="4" t="s">
         <v>20</v>
       </c>
     </row>
@@ -9901,15 +9911,15 @@
       <c r="A13" t="s">
         <v>17</v>
       </c>
-      <c r="B13" s="6">
+      <c r="B13" s="5">
         <f>SUMIFS('RAG Comparison'!$D:$D,'RAG Comparison'!$A:$A,$A13,'RAG Comparison'!$B:$B,B$12)</f>
         <v>0.98670000000000002</v>
       </c>
-      <c r="C13" s="6">
+      <c r="C13" s="5">
         <f>SUMIFS('RAG Comparison'!$D:$D,'RAG Comparison'!$A:$A,$A13,'RAG Comparison'!$B:$B,C$12)</f>
         <v>0.9133</v>
       </c>
-      <c r="D13" s="6">
+      <c r="D13" s="5">
         <f>SUMIFS('RAG Comparison'!$D:$D,'RAG Comparison'!$A:$A,$A13,'RAG Comparison'!$B:$B,D$12)</f>
         <v>0.92669999999999997</v>
       </c>
@@ -9918,15 +9928,15 @@
       <c r="A14" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="6">
+      <c r="B14" s="5">
         <f>SUMIFS('RAG Comparison'!$D:$D,'RAG Comparison'!$A:$A,$A14,'RAG Comparison'!$B:$B,B$12)</f>
         <v>0.9163</v>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="5">
         <f>SUMIFS('RAG Comparison'!$D:$D,'RAG Comparison'!$A:$A,$A14,'RAG Comparison'!$B:$B,C$12)</f>
         <v>0.90869999999999995</v>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="5">
         <f>SUMIFS('RAG Comparison'!$D:$D,'RAG Comparison'!$A:$A,$A14,'RAG Comparison'!$B:$B,D$12)</f>
         <v>0.91259999999999997</v>
       </c>
@@ -9935,15 +9945,15 @@
       <c r="A15" t="s">
         <v>22</v>
       </c>
-      <c r="B15" s="6">
+      <c r="B15" s="5">
         <f>SUMIFS('RAG Comparison'!$D:$D,'RAG Comparison'!$A:$A,$A15,'RAG Comparison'!$B:$B,B$12)</f>
         <v>0.9667</v>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="5">
         <f>SUMIFS('RAG Comparison'!$D:$D,'RAG Comparison'!$A:$A,$A15,'RAG Comparison'!$B:$B,C$12)</f>
         <v>0.66</v>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="5">
         <f>SUMIFS('RAG Comparison'!$D:$D,'RAG Comparison'!$A:$A,$A15,'RAG Comparison'!$B:$B,D$12)</f>
         <v>0.76670000000000005</v>
       </c>
@@ -9952,35 +9962,35 @@
       <c r="A16" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="6">
+      <c r="B16" s="5">
         <f>SUMIFS('RAG Comparison'!$D:$D,'RAG Comparison'!$A:$A,$A16,'RAG Comparison'!$B:$B,B$12)</f>
         <v>0.9667</v>
       </c>
-      <c r="C16" s="6">
+      <c r="C16" s="5">
         <f>SUMIFS('RAG Comparison'!$D:$D,'RAG Comparison'!$A:$A,$A16,'RAG Comparison'!$B:$B,C$12)</f>
         <v>0.95330000000000004</v>
       </c>
-      <c r="D16" s="6">
+      <c r="D16" s="5">
         <f>SUMIFS('RAG Comparison'!$D:$D,'RAG Comparison'!$A:$A,$A16,'RAG Comparison'!$B:$B,D$12)</f>
         <v>0.92669999999999997</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="4" t="s">
         <v>20</v>
       </c>
     </row>
@@ -9988,15 +9998,15 @@
       <c r="A21" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="6">
+      <c r="B21" s="5">
         <f>SUMIFS('RAG Comparison'!$F:$F,'RAG Comparison'!$A:$A,$A21,'RAG Comparison'!$B:$B,B$20)</f>
         <v>0.9</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="5">
         <f>SUMIFS('RAG Comparison'!$F:$F,'RAG Comparison'!$A:$A,$A21,'RAG Comparison'!$B:$B,C$20)</f>
         <v>0.86</v>
       </c>
-      <c r="D21" s="6">
+      <c r="D21" s="5">
         <f>SUMIFS('RAG Comparison'!$F:$F,'RAG Comparison'!$A:$A,$A21,'RAG Comparison'!$B:$B,D$20)</f>
         <v>0.89</v>
       </c>
@@ -10005,15 +10015,15 @@
       <c r="A22" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="6">
+      <c r="B22" s="5">
         <f>SUMIFS('RAG Comparison'!$F:$F,'RAG Comparison'!$A:$A,$A22,'RAG Comparison'!$B:$B,B$20)</f>
         <v>0.93</v>
       </c>
-      <c r="C22" s="6">
+      <c r="C22" s="5">
         <f>SUMIFS('RAG Comparison'!$F:$F,'RAG Comparison'!$A:$A,$A22,'RAG Comparison'!$B:$B,C$20)</f>
         <v>0.93</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D22" s="5">
         <f>SUMIFS('RAG Comparison'!$F:$F,'RAG Comparison'!$A:$A,$A22,'RAG Comparison'!$B:$B,D$20)</f>
         <v>0.96</v>
       </c>
@@ -10022,15 +10032,15 @@
       <c r="A23" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="6">
+      <c r="B23" s="5">
         <f>SUMIFS('RAG Comparison'!$F:$F,'RAG Comparison'!$A:$A,$A23,'RAG Comparison'!$B:$B,B$20)</f>
         <v>0.94</v>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="5">
         <f>SUMIFS('RAG Comparison'!$F:$F,'RAG Comparison'!$A:$A,$A23,'RAG Comparison'!$B:$B,C$20)</f>
         <v>0.77</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="5">
         <f>SUMIFS('RAG Comparison'!$F:$F,'RAG Comparison'!$A:$A,$A23,'RAG Comparison'!$B:$B,D$20)</f>
         <v>0.83</v>
       </c>
@@ -10039,35 +10049,35 @@
       <c r="A24" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="6">
+      <c r="B24" s="5">
         <f>SUMIFS('RAG Comparison'!$F:$F,'RAG Comparison'!$A:$A,$A24,'RAG Comparison'!$B:$B,B$20)</f>
         <v>0.96</v>
       </c>
-      <c r="C24" s="6">
+      <c r="C24" s="5">
         <f>SUMIFS('RAG Comparison'!$F:$F,'RAG Comparison'!$A:$A,$A24,'RAG Comparison'!$B:$B,C$20)</f>
         <v>0.96</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="5">
         <f>SUMIFS('RAG Comparison'!$F:$F,'RAG Comparison'!$A:$A,$A24,'RAG Comparison'!$B:$B,D$20)</f>
         <v>0.94</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="3" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="D28" s="4" t="s">
         <v>20</v>
       </c>
     </row>
@@ -10075,15 +10085,15 @@
       <c r="A29" t="s">
         <v>17</v>
       </c>
-      <c r="B29" s="7">
+      <c r="B29" s="6">
         <f>SUMIFS('RAG Comparison'!$E:$E,'RAG Comparison'!$A:$A,$A29,'RAG Comparison'!$B:$B,B$28)</f>
         <v>5</v>
       </c>
-      <c r="C29" s="7">
+      <c r="C29" s="6">
         <f>SUMIFS('RAG Comparison'!$E:$E,'RAG Comparison'!$A:$A,$A29,'RAG Comparison'!$B:$B,C$28)</f>
         <v>4.8</v>
       </c>
-      <c r="D29" s="7">
+      <c r="D29" s="6">
         <f>SUMIFS('RAG Comparison'!$E:$E,'RAG Comparison'!$A:$A,$A29,'RAG Comparison'!$B:$B,D$28)</f>
         <v>4.84</v>
       </c>
@@ -10092,15 +10102,15 @@
       <c r="A30" t="s">
         <v>21</v>
       </c>
-      <c r="B30" s="7">
+      <c r="B30" s="6">
         <f>SUMIFS('RAG Comparison'!$E:$E,'RAG Comparison'!$A:$A,$A30,'RAG Comparison'!$B:$B,B$28)</f>
         <v>5</v>
       </c>
-      <c r="C30" s="7">
+      <c r="C30" s="6">
         <f>SUMIFS('RAG Comparison'!$E:$E,'RAG Comparison'!$A:$A,$A30,'RAG Comparison'!$B:$B,C$28)</f>
         <v>4.8</v>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="6">
         <f>SUMIFS('RAG Comparison'!$E:$E,'RAG Comparison'!$A:$A,$A30,'RAG Comparison'!$B:$B,D$28)</f>
         <v>5</v>
       </c>
@@ -10109,15 +10119,15 @@
       <c r="A31" t="s">
         <v>22</v>
       </c>
-      <c r="B31" s="7">
+      <c r="B31" s="6">
         <f>SUMIFS('RAG Comparison'!$E:$E,'RAG Comparison'!$A:$A,$A31,'RAG Comparison'!$B:$B,B$28)</f>
         <v>4.96</v>
       </c>
-      <c r="C31" s="7">
+      <c r="C31" s="6">
         <f>SUMIFS('RAG Comparison'!$E:$E,'RAG Comparison'!$A:$A,$A31,'RAG Comparison'!$B:$B,C$28)</f>
         <v>4.6399999999999997</v>
       </c>
-      <c r="D31" s="7">
+      <c r="D31" s="6">
         <f>SUMIFS('RAG Comparison'!$E:$E,'RAG Comparison'!$A:$A,$A31,'RAG Comparison'!$B:$B,D$28)</f>
         <v>4.72</v>
       </c>
@@ -10126,35 +10136,35 @@
       <c r="A32" t="s">
         <v>23</v>
       </c>
-      <c r="B32" s="7">
+      <c r="B32" s="6">
         <f>SUMIFS('RAG Comparison'!$E:$E,'RAG Comparison'!$A:$A,$A32,'RAG Comparison'!$B:$B,B$28)</f>
         <v>5</v>
       </c>
-      <c r="C32" s="7">
+      <c r="C32" s="6">
         <f>SUMIFS('RAG Comparison'!$E:$E,'RAG Comparison'!$A:$A,$A32,'RAG Comparison'!$B:$B,C$28)</f>
         <v>5</v>
       </c>
-      <c r="D32" s="7">
+      <c r="D32" s="6">
         <f>SUMIFS('RAG Comparison'!$E:$E,'RAG Comparison'!$A:$A,$A32,'RAG Comparison'!$B:$B,D$28)</f>
         <v>4.96</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A35" s="4" t="s">
+      <c r="A35" s="3" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="5" t="s">
+      <c r="A36" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="C36" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="D36" s="4" t="s">
         <v>20</v>
       </c>
     </row>
@@ -10162,15 +10172,15 @@
       <c r="A37" t="s">
         <v>17</v>
       </c>
-      <c r="B37" s="6">
+      <c r="B37" s="5">
         <f>SUMIFS('RAG Comparison'!$G:$G,'RAG Comparison'!$A:$A,$A37,'RAG Comparison'!$B:$B,B$36)</f>
         <v>0.48159999999999997</v>
       </c>
-      <c r="C37" s="6">
+      <c r="C37" s="5">
         <f>SUMIFS('RAG Comparison'!$G:$G,'RAG Comparison'!$A:$A,$A37,'RAG Comparison'!$B:$B,C$36)</f>
         <v>0.45760000000000001</v>
       </c>
-      <c r="D37" s="6">
+      <c r="D37" s="5">
         <f>SUMIFS('RAG Comparison'!$G:$G,'RAG Comparison'!$A:$A,$A37,'RAG Comparison'!$B:$B,D$36)</f>
         <v>0.48080000000000001</v>
       </c>
@@ -10179,15 +10189,15 @@
       <c r="A38" t="s">
         <v>21</v>
       </c>
-      <c r="B38" s="6">
+      <c r="B38" s="5">
         <f>SUMIFS('RAG Comparison'!$G:$G,'RAG Comparison'!$A:$A,$A38,'RAG Comparison'!$B:$B,B$36)</f>
         <v>0.48359999999999997</v>
       </c>
-      <c r="C38" s="6">
+      <c r="C38" s="5">
         <f>SUMIFS('RAG Comparison'!$G:$G,'RAG Comparison'!$A:$A,$A38,'RAG Comparison'!$B:$B,C$36)</f>
         <v>0.48799999999999999</v>
       </c>
-      <c r="D38" s="6">
+      <c r="D38" s="5">
         <f>SUMIFS('RAG Comparison'!$G:$G,'RAG Comparison'!$A:$A,$A38,'RAG Comparison'!$B:$B,D$36)</f>
         <v>0.50439999999999996</v>
       </c>
@@ -10196,15 +10206,15 @@
       <c r="A39" t="s">
         <v>22</v>
       </c>
-      <c r="B39" s="6">
+      <c r="B39" s="5">
         <f>SUMIFS('RAG Comparison'!$G:$G,'RAG Comparison'!$A:$A,$A39,'RAG Comparison'!$B:$B,B$36)</f>
         <v>0.4108</v>
       </c>
-      <c r="C39" s="6">
+      <c r="C39" s="5">
         <f>SUMIFS('RAG Comparison'!$G:$G,'RAG Comparison'!$A:$A,$A39,'RAG Comparison'!$B:$B,C$36)</f>
         <v>0.38319999999999999</v>
       </c>
-      <c r="D39" s="6">
+      <c r="D39" s="5">
         <f>SUMIFS('RAG Comparison'!$G:$G,'RAG Comparison'!$A:$A,$A39,'RAG Comparison'!$B:$B,D$36)</f>
         <v>0.4052</v>
       </c>
@@ -10213,35 +10223,35 @@
       <c r="A40" t="s">
         <v>23</v>
       </c>
-      <c r="B40" s="6">
+      <c r="B40" s="5">
         <f>SUMIFS('RAG Comparison'!$G:$G,'RAG Comparison'!$A:$A,$A40,'RAG Comparison'!$B:$B,B$36)</f>
         <v>0.59160000000000001</v>
       </c>
-      <c r="C40" s="6">
+      <c r="C40" s="5">
         <f>SUMIFS('RAG Comparison'!$G:$G,'RAG Comparison'!$A:$A,$A40,'RAG Comparison'!$B:$B,C$36)</f>
         <v>0.59040000000000004</v>
       </c>
-      <c r="D40" s="6">
+      <c r="D40" s="5">
         <f>SUMIFS('RAG Comparison'!$G:$G,'RAG Comparison'!$A:$A,$A40,'RAG Comparison'!$B:$B,D$36)</f>
         <v>0.61439999999999995</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A43" s="4" t="s">
+      <c r="A43" s="3" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="5" t="s">
+      <c r="A44" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B44" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="C44" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D44" s="5" t="s">
+      <c r="D44" s="4" t="s">
         <v>20</v>
       </c>
     </row>
@@ -10249,15 +10259,15 @@
       <c r="A45" t="s">
         <v>17</v>
       </c>
-      <c r="B45" s="8">
+      <c r="B45" s="7">
         <f>SUMIFS('RAG Comparison'!$L:$L,'RAG Comparison'!$A:$A,$A45,'RAG Comparison'!$B:$B,B$44)</f>
         <v>5.8500000000000002E-4</v>
       </c>
-      <c r="C45" s="8">
+      <c r="C45" s="7">
         <f>SUMIFS('RAG Comparison'!$L:$L,'RAG Comparison'!$A:$A,$A45,'RAG Comparison'!$B:$B,C$44)</f>
         <v>7.27E-4</v>
       </c>
-      <c r="D45" s="8">
+      <c r="D45" s="7">
         <f>SUMIFS('RAG Comparison'!$L:$L,'RAG Comparison'!$A:$A,$A45,'RAG Comparison'!$B:$B,D$44)</f>
         <v>7.67E-4</v>
       </c>
@@ -10266,15 +10276,15 @@
       <c r="A46" t="s">
         <v>21</v>
       </c>
-      <c r="B46" s="8">
+      <c r="B46" s="7">
         <f>SUMIFS('RAG Comparison'!$L:$L,'RAG Comparison'!$A:$A,$A46,'RAG Comparison'!$B:$B,B$44)</f>
         <v>9.68E-4</v>
       </c>
-      <c r="C46" s="8">
+      <c r="C46" s="7">
         <f>SUMIFS('RAG Comparison'!$L:$L,'RAG Comparison'!$A:$A,$A46,'RAG Comparison'!$B:$B,C$44)</f>
         <v>8.34E-4</v>
       </c>
-      <c r="D46" s="8">
+      <c r="D46" s="7">
         <f>SUMIFS('RAG Comparison'!$L:$L,'RAG Comparison'!$A:$A,$A46,'RAG Comparison'!$B:$B,D$44)</f>
         <v>8.9599999999999999E-4</v>
       </c>
@@ -10283,15 +10293,15 @@
       <c r="A47" t="s">
         <v>22</v>
       </c>
-      <c r="B47" s="8">
+      <c r="B47" s="7">
         <f>SUMIFS('RAG Comparison'!$L:$L,'RAG Comparison'!$A:$A,$A47,'RAG Comparison'!$B:$B,B$44)</f>
         <v>1.024E-3</v>
       </c>
-      <c r="C47" s="8">
+      <c r="C47" s="7">
         <f>SUMIFS('RAG Comparison'!$L:$L,'RAG Comparison'!$A:$A,$A47,'RAG Comparison'!$B:$B,C$44)</f>
         <v>8.61E-4</v>
       </c>
-      <c r="D47" s="8">
+      <c r="D47" s="7">
         <f>SUMIFS('RAG Comparison'!$L:$L,'RAG Comparison'!$A:$A,$A47,'RAG Comparison'!$B:$B,D$44)</f>
         <v>9.19E-4</v>
       </c>
@@ -10300,35 +10310,35 @@
       <c r="A48" t="s">
         <v>23</v>
       </c>
-      <c r="B48" s="8">
+      <c r="B48" s="7">
         <f>SUMIFS('RAG Comparison'!$L:$L,'RAG Comparison'!$A:$A,$A48,'RAG Comparison'!$B:$B,B$44)</f>
         <v>9.01E-4</v>
       </c>
-      <c r="C48" s="8">
+      <c r="C48" s="7">
         <f>SUMIFS('RAG Comparison'!$L:$L,'RAG Comparison'!$A:$A,$A48,'RAG Comparison'!$B:$B,C$44)</f>
         <v>8.4500000000000005E-4</v>
       </c>
-      <c r="D48" s="8">
+      <c r="D48" s="7">
         <f>SUMIFS('RAG Comparison'!$L:$L,'RAG Comparison'!$A:$A,$A48,'RAG Comparison'!$B:$B,D$44)</f>
         <v>8.6899999999999998E-4</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A51" s="4" t="s">
+      <c r="A51" s="3" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="5" t="s">
+      <c r="A52" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B52" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="C52" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D52" s="5" t="s">
+      <c r="D52" s="4" t="s">
         <v>20</v>
       </c>
     </row>
@@ -10336,15 +10346,15 @@
       <c r="A53" t="s">
         <v>17</v>
       </c>
-      <c r="B53" s="8">
+      <c r="B53" s="7">
         <f>SUMIFS('RAG Comparison'!$P:$P,'RAG Comparison'!$A:$A,$A53,'RAG Comparison'!$B:$B,B$52)</f>
         <v>5.8500000000000002E-4</v>
       </c>
-      <c r="C53" s="8">
+      <c r="C53" s="7">
         <f>SUMIFS('RAG Comparison'!$P:$P,'RAG Comparison'!$A:$A,$A53,'RAG Comparison'!$B:$B,C$52)</f>
         <v>7.27E-4</v>
       </c>
-      <c r="D53" s="8">
+      <c r="D53" s="7">
         <f>SUMIFS('RAG Comparison'!$P:$P,'RAG Comparison'!$A:$A,$A53,'RAG Comparison'!$B:$B,D$52)</f>
         <v>7.67E-4</v>
       </c>
@@ -10353,15 +10363,15 @@
       <c r="A54" t="s">
         <v>21</v>
       </c>
-      <c r="B54" s="8">
+      <c r="B54" s="7">
         <f>SUMIFS('RAG Comparison'!$P:$P,'RAG Comparison'!$A:$A,$A54,'RAG Comparison'!$B:$B,B$52)</f>
         <v>9.68E-4</v>
       </c>
-      <c r="C54" s="8">
+      <c r="C54" s="7">
         <f>SUMIFS('RAG Comparison'!$P:$P,'RAG Comparison'!$A:$A,$A54,'RAG Comparison'!$B:$B,C$52)</f>
         <v>8.34E-4</v>
       </c>
-      <c r="D54" s="8">
+      <c r="D54" s="7">
         <f>SUMIFS('RAG Comparison'!$P:$P,'RAG Comparison'!$A:$A,$A54,'RAG Comparison'!$B:$B,D$52)</f>
         <v>8.9599999999999999E-4</v>
       </c>
@@ -10370,15 +10380,15 @@
       <c r="A55" t="s">
         <v>22</v>
       </c>
-      <c r="B55" s="8">
+      <c r="B55" s="7">
         <f>SUMIFS('RAG Comparison'!$P:$P,'RAG Comparison'!$A:$A,$A55,'RAG Comparison'!$B:$B,B$52)</f>
         <v>1.024E-3</v>
       </c>
-      <c r="C55" s="8">
+      <c r="C55" s="7">
         <f>SUMIFS('RAG Comparison'!$P:$P,'RAG Comparison'!$A:$A,$A55,'RAG Comparison'!$B:$B,C$52)</f>
         <v>8.61E-4</v>
       </c>
-      <c r="D55" s="8">
+      <c r="D55" s="7">
         <f>SUMIFS('RAG Comparison'!$P:$P,'RAG Comparison'!$A:$A,$A55,'RAG Comparison'!$B:$B,D$52)</f>
         <v>9.19E-4</v>
       </c>
@@ -10387,35 +10397,35 @@
       <c r="A56" t="s">
         <v>23</v>
       </c>
-      <c r="B56" s="8">
+      <c r="B56" s="7">
         <f>SUMIFS('RAG Comparison'!$P:$P,'RAG Comparison'!$A:$A,$A56,'RAG Comparison'!$B:$B,B$52)</f>
         <v>9.01E-4</v>
       </c>
-      <c r="C56" s="8">
+      <c r="C56" s="7">
         <f>SUMIFS('RAG Comparison'!$P:$P,'RAG Comparison'!$A:$A,$A56,'RAG Comparison'!$B:$B,C$52)</f>
         <v>8.4500000000000005E-4</v>
       </c>
-      <c r="D56" s="8">
+      <c r="D56" s="7">
         <f>SUMIFS('RAG Comparison'!$P:$P,'RAG Comparison'!$A:$A,$A56,'RAG Comparison'!$B:$B,D$52)</f>
         <v>8.6899999999999998E-4</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A59" s="4" t="s">
+      <c r="A59" s="3" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="5" t="s">
+      <c r="A60" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="B60" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C60" s="5" t="s">
+      <c r="C60" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D60" s="5" t="s">
+      <c r="D60" s="4" t="s">
         <v>20</v>
       </c>
     </row>
@@ -10423,15 +10433,15 @@
       <c r="A61" t="s">
         <v>17</v>
       </c>
-      <c r="B61" s="9">
+      <c r="B61" s="8">
         <f>SUMIFS('RAG Comparison'!$M:$M,'RAG Comparison'!$A:$A,$A61,'RAG Comparison'!$B:$B,B$60)</f>
         <v>23163.68</v>
       </c>
-      <c r="C61" s="9">
+      <c r="C61" s="8">
         <f>SUMIFS('RAG Comparison'!$M:$M,'RAG Comparison'!$A:$A,$A61,'RAG Comparison'!$B:$B,C$60)</f>
         <v>2154</v>
       </c>
-      <c r="D61" s="9">
+      <c r="D61" s="8">
         <f>SUMIFS('RAG Comparison'!$M:$M,'RAG Comparison'!$A:$A,$A61,'RAG Comparison'!$B:$B,D$60)</f>
         <v>2287.6799999999998</v>
       </c>
@@ -10440,15 +10450,15 @@
       <c r="A62" t="s">
         <v>21</v>
       </c>
-      <c r="B62" s="9">
+      <c r="B62" s="8">
         <f>SUMIFS('RAG Comparison'!$M:$M,'RAG Comparison'!$A:$A,$A62,'RAG Comparison'!$B:$B,B$60)</f>
         <v>27078.880000000001</v>
       </c>
-      <c r="C62" s="9">
+      <c r="C62" s="8">
         <f>SUMIFS('RAG Comparison'!$M:$M,'RAG Comparison'!$A:$A,$A62,'RAG Comparison'!$B:$B,C$60)</f>
         <v>2297.6</v>
       </c>
-      <c r="D62" s="9">
+      <c r="D62" s="8">
         <f>SUMIFS('RAG Comparison'!$M:$M,'RAG Comparison'!$A:$A,$A62,'RAG Comparison'!$B:$B,D$60)</f>
         <v>2416.88</v>
       </c>
@@ -10457,15 +10467,15 @@
       <c r="A63" t="s">
         <v>22</v>
       </c>
-      <c r="B63" s="9">
+      <c r="B63" s="8">
         <f>SUMIFS('RAG Comparison'!$M:$M,'RAG Comparison'!$A:$A,$A63,'RAG Comparison'!$B:$B,B$60)</f>
         <v>26697.84</v>
       </c>
-      <c r="C63" s="9">
+      <c r="C63" s="8">
         <f>SUMIFS('RAG Comparison'!$M:$M,'RAG Comparison'!$A:$A,$A63,'RAG Comparison'!$B:$B,C$60)</f>
         <v>2302.16</v>
       </c>
-      <c r="D63" s="9">
+      <c r="D63" s="8">
         <f>SUMIFS('RAG Comparison'!$M:$M,'RAG Comparison'!$A:$A,$A63,'RAG Comparison'!$B:$B,D$60)</f>
         <v>2438.08</v>
       </c>
@@ -10474,15 +10484,15 @@
       <c r="A64" t="s">
         <v>23</v>
       </c>
-      <c r="B64" s="9">
+      <c r="B64" s="8">
         <f>SUMIFS('RAG Comparison'!$M:$M,'RAG Comparison'!$A:$A,$A64,'RAG Comparison'!$B:$B,B$60)</f>
         <v>29899.4</v>
       </c>
-      <c r="C64" s="9">
+      <c r="C64" s="8">
         <f>SUMIFS('RAG Comparison'!$M:$M,'RAG Comparison'!$A:$A,$A64,'RAG Comparison'!$B:$B,C$60)</f>
         <v>2444.88</v>
       </c>
-      <c r="D64" s="9">
+      <c r="D64" s="8">
         <f>SUMIFS('RAG Comparison'!$M:$M,'RAG Comparison'!$A:$A,$A64,'RAG Comparison'!$B:$B,D$60)</f>
         <v>2483.96</v>
       </c>

</xml_diff>